<commit_message>
Added Precedence Graph for SAT and MaxSAT
</commit_message>
<xml_diff>
--- a/results/2026-04-04-SAT-initial-synchronous-heuristic/Tóm tắt kết quả.xlsx
+++ b/results/2026-04-04-SAT-initial-synchronous-heuristic/Tóm tắt kết quả.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\maxsattrainscheduling\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\maxsattrainscheduling\results\2026-04-04-SAT-initial-synchronous-heuristic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CDCACDFB-0FFD-453A-B4C0-9B092FA06188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DAA7DA18-1B33-4F62-A473-65B42A627968}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="17715"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -75,7 +74,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -941,49 +940,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
@@ -995,13 +958,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
@@ -1010,9 +970,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="41" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="43" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1027,17 +984,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="51" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="43" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="52" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="42" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="53" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="58" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="59" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="1" applyBorder="1"/>
@@ -1049,6 +1001,56 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="53" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="43" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="52" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="20% - Accent5" xfId="1" builtinId="46"/>
@@ -1363,402 +1365,403 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{287D06EE-AE05-470D-8219-850D6C5ED8C5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.21875" customWidth="1"/>
-    <col min="7" max="7" width="9.6640625" customWidth="1"/>
-    <col min="8" max="8" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="63" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="65" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="75"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="56"/>
     </row>
-    <row r="2" spans="1:9" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="5"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="7" t="s">
+    <row r="2" spans="1:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="64"/>
+      <c r="B2" s="66"/>
+      <c r="C2" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="9" t="s">
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="72" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="8"/>
-      <c r="H2" s="10"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="73"/>
     </row>
-    <row r="3" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="5"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="12" t="s">
+    <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="64"/>
+      <c r="B3" s="67"/>
+      <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="76" t="s">
+      <c r="H3" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="75"/>
+      <c r="I3" s="56"/>
     </row>
-    <row r="4" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="60" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="19">
+      <c r="C4" s="7">
         <v>11763.28</v>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="8">
         <v>47001.25</v>
       </c>
-      <c r="E4" s="21">
-        <v>1879.4179999999999</v>
-      </c>
-      <c r="F4" s="22">
+      <c r="E4" s="9">
+        <v>413.90940000000001</v>
+      </c>
+      <c r="F4" s="10">
         <v>22</v>
       </c>
-      <c r="G4" s="23">
+      <c r="G4" s="11">
         <v>15</v>
       </c>
-      <c r="H4" s="24">
+      <c r="H4" s="12">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="17"/>
-      <c r="B5" s="25" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="60"/>
+      <c r="B5" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="14">
         <v>23035.61</v>
       </c>
-      <c r="D5" s="27">
+      <c r="D5" s="15">
         <v>85001.46</v>
       </c>
-      <c r="E5" s="28">
-        <v>31077.13</v>
-      </c>
-      <c r="F5" s="29">
+      <c r="E5" s="16">
+        <v>16095.81</v>
+      </c>
+      <c r="F5" s="74">
         <v>20</v>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="15">
         <v>7</v>
       </c>
-      <c r="H5" s="77">
+      <c r="H5" s="58">
+        <v>21</v>
+      </c>
+      <c r="I5" s="56"/>
+    </row>
+    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="60"/>
+      <c r="B6" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="18">
+        <v>42557.14</v>
+      </c>
+      <c r="D6" s="19">
+        <v>90078.45</v>
+      </c>
+      <c r="E6" s="20">
+        <v>26595.52</v>
+      </c>
+      <c r="F6" s="75">
+        <v>18</v>
+      </c>
+      <c r="G6" s="19">
+        <v>6</v>
+      </c>
+      <c r="H6" s="59">
         <v>20</v>
       </c>
-      <c r="I5" s="75"/>
     </row>
-    <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="17"/>
-      <c r="B6" s="30" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="31">
-        <v>42557.14</v>
-      </c>
-      <c r="D6" s="32">
-        <v>90078.45</v>
-      </c>
-      <c r="E6" s="33">
-        <v>39742.83</v>
-      </c>
-      <c r="F6" s="34">
-        <v>18</v>
-      </c>
-      <c r="G6" s="32">
-        <v>6</v>
-      </c>
-      <c r="H6" s="78">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="17"/>
-      <c r="B7" s="39" t="s">
+    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="60"/>
+      <c r="B7" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="40">
+      <c r="C7" s="25">
         <f>SUM(C4:C6)</f>
         <v>77356.03</v>
       </c>
-      <c r="D7" s="41">
+      <c r="D7" s="26">
         <f>SUM(D4:D6)</f>
         <v>222081.16000000003</v>
       </c>
-      <c r="E7" s="42">
+      <c r="E7" s="27">
         <f t="shared" ref="E7:H7" si="0">SUM(E4:E6)</f>
-        <v>72699.377999999997</v>
-      </c>
-      <c r="F7" s="74">
+        <v>43105.239399999999</v>
+      </c>
+      <c r="F7" s="55">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
-      <c r="G7" s="43">
+      <c r="G7" s="28">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="H7" s="42">
+      <c r="H7" s="27">
         <f t="shared" si="0"/>
-        <v>62</v>
-      </c>
-      <c r="I7" s="75"/>
+        <v>65</v>
+      </c>
+      <c r="I7" s="56"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="44" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="61" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="45" t="s">
+      <c r="B8" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="46">
+      <c r="C8" s="30">
         <v>18.09</v>
       </c>
-      <c r="D8" s="47">
+      <c r="D8" s="31">
         <v>10.46034</v>
       </c>
-      <c r="E8" s="48">
-        <v>27.669319999999999</v>
-      </c>
-      <c r="F8" s="49">
+      <c r="E8" s="32">
+        <v>44.266109999999998</v>
+      </c>
+      <c r="F8" s="33">
         <v>24</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="8">
         <v>24</v>
       </c>
-      <c r="H8" s="50">
+      <c r="H8" s="34">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="44"/>
-      <c r="B9" s="51" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="61"/>
+      <c r="B9" s="35" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="27">
+      <c r="C9" s="15">
         <v>10491.134309999999</v>
       </c>
-      <c r="D9" s="52">
+      <c r="D9" s="77">
         <v>7269.5829999999996</v>
       </c>
-      <c r="E9" s="28">
-        <v>11607.29</v>
-      </c>
-      <c r="F9" s="53">
+      <c r="E9" s="58">
+        <v>1719.7260000000001</v>
+      </c>
+      <c r="F9" s="37">
         <v>22</v>
       </c>
-      <c r="G9" s="52">
+      <c r="G9" s="36">
         <v>24</v>
       </c>
-      <c r="H9" s="77">
+      <c r="H9" s="58">
         <v>24</v>
       </c>
-      <c r="I9" s="75"/>
+      <c r="I9" s="56"/>
     </row>
-    <row r="10" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="44"/>
-      <c r="B10" s="54" t="s">
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="61"/>
+      <c r="B10" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="37">
+      <c r="C10" s="22">
         <v>11762.97784</v>
       </c>
-      <c r="D10" s="55">
+      <c r="D10" s="78">
         <v>5030.67</v>
       </c>
-      <c r="E10" s="38">
-        <v>8345.4470000000001</v>
-      </c>
-      <c r="F10" s="56">
+      <c r="E10" s="79">
+        <v>363.31479999999999</v>
+      </c>
+      <c r="F10" s="40">
         <v>22</v>
       </c>
-      <c r="G10" s="55">
+      <c r="G10" s="39">
         <v>24</v>
       </c>
-      <c r="H10" s="35">
-        <v>23</v>
+      <c r="H10" s="59">
+        <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="44"/>
-      <c r="B11" s="57" t="s">
+    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="61"/>
+      <c r="B11" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="40">
+      <c r="C11" s="25">
         <f>SUM(C8:C10)</f>
         <v>22272.202149999997</v>
       </c>
-      <c r="D11" s="58">
+      <c r="D11" s="80">
         <f>SUM(D8:D10)</f>
         <v>12310.713339999998</v>
       </c>
-      <c r="E11" s="59">
+      <c r="E11" s="81">
         <f t="shared" ref="E11:G11" si="1">SUM(E8:E10)</f>
-        <v>19980.406320000002</v>
-      </c>
-      <c r="F11" s="60">
+        <v>2127.3069100000002</v>
+      </c>
+      <c r="F11" s="43">
         <f t="shared" si="1"/>
         <v>68</v>
       </c>
-      <c r="G11" s="58">
+      <c r="G11" s="42">
         <f t="shared" si="1"/>
         <v>72</v>
       </c>
-      <c r="H11" s="61">
+      <c r="H11" s="76">
         <f>SUM(H8:H10)</f>
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="62" t="s">
+      <c r="B12" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="63">
+      <c r="C12" s="45">
         <v>6.3201721300000004</v>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="8">
         <v>8.4396679999999993</v>
       </c>
-      <c r="E12" s="64">
-        <v>37.37274</v>
-      </c>
-      <c r="F12" s="49">
+      <c r="E12" s="46">
+        <v>41.573369999999997</v>
+      </c>
+      <c r="F12" s="33">
         <v>24</v>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="8">
         <v>24</v>
       </c>
-      <c r="H12" s="64">
+      <c r="H12" s="46">
         <v>24</v>
       </c>
-      <c r="I12" s="75"/>
+      <c r="I12" s="56"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="17"/>
-      <c r="B13" s="65" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="60"/>
+      <c r="B13" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="26">
+      <c r="C13" s="14">
         <v>24.887712709999999</v>
       </c>
-      <c r="D13" s="27">
+      <c r="D13" s="15">
         <v>94.609719999999996</v>
       </c>
-      <c r="E13" s="28">
-        <v>129.405</v>
-      </c>
-      <c r="F13" s="53">
+      <c r="E13" s="16">
+        <v>82.702619999999996</v>
+      </c>
+      <c r="F13" s="37">
         <v>24</v>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="15">
         <v>24</v>
       </c>
-      <c r="H13" s="28">
+      <c r="H13" s="16">
         <v>24</v>
       </c>
-      <c r="I13" s="75"/>
+      <c r="I13" s="56"/>
     </row>
-    <row r="14" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="17"/>
-      <c r="B14" s="66" t="s">
+    <row r="14" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="60"/>
+      <c r="B14" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="36">
+      <c r="C14" s="21">
         <v>26.39</v>
       </c>
-      <c r="D14" s="37">
+      <c r="D14" s="22">
         <v>78.652550000000005</v>
       </c>
-      <c r="E14" s="38">
-        <v>83.226799999999997</v>
-      </c>
-      <c r="F14" s="56">
+      <c r="E14" s="23">
+        <v>88.108360000000005</v>
+      </c>
+      <c r="F14" s="40">
         <v>24</v>
       </c>
-      <c r="G14" s="37">
+      <c r="G14" s="22">
         <v>24</v>
       </c>
-      <c r="H14" s="38">
+      <c r="H14" s="23">
         <v>24</v>
       </c>
-      <c r="I14" s="75"/>
+      <c r="I14" s="56"/>
     </row>
-    <row r="15" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="67"/>
-      <c r="B15" s="68" t="s">
+    <row r="15" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="62"/>
+      <c r="B15" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="69">
+      <c r="C15" s="50">
         <f>SUM(C12:C14)</f>
         <v>57.597884839999999</v>
       </c>
-      <c r="D15" s="70">
+      <c r="D15" s="51">
         <f>SUM(D12:D14)</f>
         <v>181.70193799999998</v>
       </c>
-      <c r="E15" s="71">
+      <c r="E15" s="52">
         <f t="shared" ref="E15:H15" si="2">SUM(E12:E14)</f>
-        <v>250.00453999999999</v>
-      </c>
-      <c r="F15" s="72">
+        <v>212.38434999999998</v>
+      </c>
+      <c r="F15" s="53">
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="G15" s="70">
+      <c r="G15" s="51">
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
-      <c r="H15" s="73">
+      <c r="H15" s="54">
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="C1:H1"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="A4:A7"/>
     <mergeCell ref="A8:A11"/>
     <mergeCell ref="A12:A15"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:H1"/>
-    <mergeCell ref="C2:E2"/>
-    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>